<commit_message>
modified shcematics BOOT botton, added connector for VTX, did rough Layout
</commit_message>
<xml_diff>
--- a/Test_Board/production/board.xlsx
+++ b/Test_Board/production/board.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Saleh work and edu\Desktop\Saleh Uni\sem 7\senior year project\Flight Controller\Test_Board\production\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{236FDFF4-BF37-4B15-9854-4DB74958CEC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A225EF0-B883-4360-AA48-50B6FD026717}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{F22B7DE4-BB99-4002-BA76-D76E093DE2B2}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="103">
   <si>
     <t>Comment</t>
   </si>
@@ -317,13 +317,25 @@
   </si>
   <si>
     <t>C14663</t>
+  </si>
+  <si>
+    <t>we have</t>
+  </si>
+  <si>
+    <t>not needed</t>
+  </si>
+  <si>
+    <t>Akaki ordered</t>
+  </si>
+  <si>
+    <t>C2903476</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -458,8 +470,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="9"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="33">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -637,6 +656,18 @@
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.39997558519241921"/>
         <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC00000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -800,9 +831,15 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -1180,17 +1217,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D8FA59A-496C-4D8B-9D41-805EAF735B1D}">
-  <dimension ref="A1:D32"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14.26953125" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="38.90625" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="58.453125" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12.6328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="16384" width="8.7265625" style="1"/>
+    <col min="5" max="5" width="13.1796875" style="1" customWidth="1"/>
+    <col min="6" max="16384" width="8.7265625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1204,7 +1242,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -1214,8 +1252,11 @@
       <c r="C2" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E2" s="1" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>7</v>
       </c>
@@ -1228,8 +1269,9 @@
       <c r="D3" s="1" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E3" s="3"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>11</v>
       </c>
@@ -1242,8 +1284,9 @@
       <c r="D4" s="1" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E4" s="3"/>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>14</v>
       </c>
@@ -1256,8 +1299,9 @@
       <c r="D5" s="1" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E5" s="3"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>17</v>
       </c>
@@ -1270,8 +1314,9 @@
       <c r="D6" s="1" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E6" s="3"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>21</v>
       </c>
@@ -1281,8 +1326,11 @@
       <c r="C7" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E7" s="1" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>23</v>
       </c>
@@ -1292,8 +1340,11 @@
       <c r="C8" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E8" s="1" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>26</v>
       </c>
@@ -1303,8 +1354,11 @@
       <c r="C9" s="1" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E9" s="1" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>29</v>
       </c>
@@ -1314,8 +1368,11 @@
       <c r="C10" s="1" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E10" s="1" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>32</v>
       </c>
@@ -1325,8 +1382,11 @@
       <c r="C11" s="1" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E11" s="1" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" s="1">
         <v>0</v>
       </c>
@@ -1339,8 +1399,9 @@
       <c r="D12" s="1" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E12" s="3"/>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" s="1">
         <v>0.1</v>
       </c>
@@ -1350,8 +1411,12 @@
       <c r="C13" s="1" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="D13" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="E13" s="3"/>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>40</v>
       </c>
@@ -1364,8 +1429,9 @@
       <c r="D14" s="1" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E14" s="3"/>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>44</v>
       </c>
@@ -1375,8 +1441,11 @@
       <c r="C15" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E15" s="1" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>46</v>
       </c>
@@ -1386,8 +1455,11 @@
       <c r="C16" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E16" s="1" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>48</v>
       </c>
@@ -1400,8 +1472,9 @@
       <c r="D17" s="1" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E17" s="3"/>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>52</v>
       </c>
@@ -1411,8 +1484,11 @@
       <c r="C18" s="1" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E18" s="1" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>55</v>
       </c>
@@ -1422,8 +1498,9 @@
       <c r="C19" s="1" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E19" s="2"/>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>58</v>
       </c>
@@ -1436,8 +1513,9 @@
       <c r="D20" s="1" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E20" s="3"/>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>62</v>
       </c>
@@ -1450,8 +1528,9 @@
       <c r="D21" s="1" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E21" s="2"/>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>66</v>
       </c>
@@ -1464,8 +1543,9 @@
       <c r="D22" s="1" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E22" s="2"/>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>70</v>
       </c>
@@ -1478,8 +1558,9 @@
       <c r="D23" s="1" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E23" s="3"/>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>73</v>
       </c>
@@ -1492,8 +1573,9 @@
       <c r="D24" s="1" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E24" s="3"/>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>76</v>
       </c>
@@ -1506,8 +1588,9 @@
       <c r="D25" s="1" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E25" s="3"/>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>79</v>
       </c>
@@ -1520,8 +1603,9 @@
       <c r="D26" s="1" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E26" s="3"/>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" s="1">
         <v>22</v>
       </c>
@@ -1534,8 +1618,9 @@
       <c r="D27" s="1" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E27" s="3"/>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
         <v>84</v>
       </c>
@@ -1548,8 +1633,9 @@
       <c r="D28" s="1" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E28" s="3"/>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
         <v>88</v>
       </c>
@@ -1559,8 +1645,11 @@
       <c r="C29" s="1" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E29" s="1" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
         <v>91</v>
       </c>
@@ -1573,8 +1662,9 @@
       <c r="D30" s="1" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E30" s="3"/>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" s="1">
         <v>330</v>
       </c>
@@ -1587,8 +1677,9 @@
       <c r="D31" s="1" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E31" s="3"/>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>96</v>
       </c>
@@ -1601,6 +1692,7 @@
       <c r="D32" s="1" t="s">
         <v>98</v>
       </c>
+      <c r="E32" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>